<commit_message>
modified:   M8Prog laravel Planning.xlsx
</commit_message>
<xml_diff>
--- a/M8Prog laravel Planning.xlsx
+++ b/M8Prog laravel Planning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mediacollegeamsterdam-my.sharepoint.com/personal/d_javorac_ma-web_nl/Documents/doc/lessen/cohort25/M8prog Lara/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="172" documentId="13_ncr:1_{99998950-EF90-4155-970D-2963A3151F72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0A4DA9A-36B0-45A9-83BF-53412C6A601F}"/>
+  <xr:revisionPtr revIDLastSave="174" documentId="13_ncr:1_{99998950-EF90-4155-970D-2963A3151F72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD73E92E-C98A-4383-8644-8E3492A62546}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="planning" sheetId="4" r:id="rId1"/>
@@ -1072,13 +1072,13 @@
       <c r="C12" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -1424,6 +1424,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="23f2e982-2831-4f7d-9473-a432dcec5614">
@@ -1431,15 +1440,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1462,26 +1462,26 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8BF8ACB-D628-4A39-B9AE-0F76DFA6057D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFE21724-5601-41C0-B593-F4FF612662E6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="9990b2e4-f671-45e9-a507-7e01c19989ed"/>
-    <ds:schemaRef ds:uri="23f2e982-2831-4f7d-9473-a432dcec5614"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFE21724-5601-41C0-B593-F4FF612662E6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8BF8ACB-D628-4A39-B9AE-0F76DFA6057D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="9990b2e4-f671-45e9-a507-7e01c19989ed"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="23f2e982-2831-4f7d-9473-a432dcec5614"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>